<commit_message>
chore: update news radar report 2026-09-09
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-09-09.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-09-09.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,54 +446,1161 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Benefits Brokers Must Adopt New Strategies to Manage Escalating Employer Health Care Costs</t>
+          <t>Employers Health and Judi Health Partner to Launch StarkRx Modular PBM Solution</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rising employer healthcare costs are forcing benefits brokers to rethink traditional advisory models and adopt innovative cost-containment strategies. This shift matters because self-funded employers increasingly demand proactive solutions to combat surging pharmacy and medical expenses without compromising employee care. For RxBenefits and its partners, this environment creates a prime opportunity to position transparent pharmacy benefit management alternatives as an essential component of the modern broker playbook.</t>
+          <t>Employers Health and Judi Health have collaborated to introduce StarkRx, a new modular pharmacy benefit management solution designed to give self-funded employers greater flexibility and control over their plan designs. This partnership matters because it addresses growing employer demand for transparent, customizable alternatives to traditional PBM models amidst rising healthcare costs. For businesses, this development signals an industry shift toward modular solutions, enabling organizations to better manage specialty drug spend and optimize overall benefit performance.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Insurance Business</t>
+          <t>Knoxville News Sentinel</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Wed, 09 Sep 2026 01:28:45 GMT</t>
+          <t>Tue, 08 Sep 2026 15:41:42 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPbWo1WVBBY01CSkpGdXkzUEUweHFxcnRkaVQxOC1rWGJDSVpzNUVFWkFQdzNrRmJOQV9PdVM2OE9DYVlpcVB5bEh2MV9UeEtVaTdNcGFmeERBMjJNT2VMZkxFSVFCU0xjZlpNS1NITDRwcjdyRFRtUk9jMVpFNTgtX0x6QlRFTkhhelRZWkZiNjBpbW5JME5aTWpseU0zMldPcU9xQmk2UnQ0RG5VUms2NUNhY0RJYW5GbkxVYnB4UV8tOFI5Smd5WW1B?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOTGphd0xkSlA5dFFMLWhIU0ZMUjVncWY0T2FTRllpM1MwMEwxWFRFc2FkQ1RTWmRDS2RyT0ZTalVyMjhwLWJUdTlUOGJXTGhnaTVPNzRUSl9rNUZTTmtHWi1fOFZ4Wmc5OF8zMFJwOGp2TXA4dmlOcGZmRUFGVzI3SEJ0ZE5MSWkxd1N0aTBOelcwNjNsZHRnNFZFUFJack8ySEpNb0hVdWpvbUJQQTdkaDhudTJiRUxE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Model Optimal Care Introduces AI Platform Designed Specifically for Self-Funded Health Plans</t>
+          <t>No Surprises Act Independent Dispute Resolution System Triggers 20% Drop in Provider Network Participation</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Model Optimal Care has launched MOC Fiduciary Intelligence, a new artificial intelligence platform built from the ground up to support self-funded employers. This tool addresses the growing need for enhanced oversight and cost management within employer-sponsored healthcare plans by leveraging AI to streamline fiduciary responsibilities. For organizations managing self-funded benefits, this technology offers a new way to navigate complex plan data, potentially improving cost containment and compliance.</t>
+          <t>Recent data reveals that the No Surprises Act's independent dispute resolution (IDR) process has led to a 20% decrease in healthcare provider network participation as physicians increasingly drop out of managed care networks over payment disputes. This trend matters because narrower provider networks shift more financial and care-access friction onto self-funded employers and their plan members, complicating network adequacy. For benefits managers and pharmacy benefit stakeholders, this signals a broader shift in provider behavior that could destabilize traditional healthcare delivery models and increase out-of-network utilization costs.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>EIN News</t>
+          <t>BenefitsPRO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tue, 08 Sep 2026 11:30:00 GMT</t>
+          <t>Tue, 08 Sep 2026 21:06:31 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxPb1V1VVJuNGtMeU4wVThsSEwweHM3NG84SVFoMmotV1lPT3JmeUtpX0lQUEFqbHZZMlJ3U2l6N29ZbGxBT2tyVnRKaTVfOFZLbFVBWlU4QV95UWowcXdrTE1Wbm96U0pFcENMRF8xTm1panhQcFVCOVc3WE5qMkt0OUVOQjBvOVhvWFF5eDBXZmV0TlYwN3dSRkZocG93bk54NXIyV0VPVFRqdFRqeENnRnowN01rSUhhWEpSUXRJUDZXVnBaRldTUG84b2hvQUloNW1vWTEyZjZfc2NIOWFoSUFwOXI1Y2tyMFd4U1RvVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNVzNEYXNtam5sQzgtNnBzczFKQWRFYkJUdlFwdjVTeG5fY05ZLW5HSmllYUFlamd0UENIWXlxTXMzdnlsNnVsRm5WWkd0ZUl0ZmdocEVVeEV3MTIyOWFpdVZLekQyYS1EU3lXOThxNVZXaVdkQWtiQVBJSTMxbWgybDNJZEpLdS1TdHJQSk5QLWNuRy1Ob09CbkZJUE1mMjY4SmF5d3dxdTZObXpYTUtVNnJoWQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Rising Healthcare And Pharmacy Costs Threaten Business Competitiveness In North Carolina</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A recent business analysis highlights how escalating healthcare and benefit expenses are undermining the economic competitiveness of employers in North Carolina, forcing companies to reevaluate their operational budgets. This trend matters because unchecked medical and drug inflation directly burdens self-funded employers who struggle to maintain robust benefits while protecting their bottom lines. For the broader industry, this signals an urgent demand for strategic cost containment, advanced PBM alternatives, and innovative pharmacy benefit management solutions that can curb rising expenditures without compromising employee health.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>The Business Journals</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 18:34:00 GMT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxObl9oV2NpOUdURjBjd3pWV3BOZ3NzWWNSN2JXQWJwY3hMbXpyQy1uUmFHN012Zm9kNm13a2JCV2E2U0JPZldIc181QXB6RzFkWGlqMjBCVzNlRUVfRnVub3NPWlo2WlNINnNBZmdvR3RPazc4azdUTkxINGM0YXFWMmZ6cDYxZ1hZLXBiYmVlYmVqajVjejg0TGR6ZmpqbHBYRHRqc0tXeGtVODA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Anthem Faces Allegations Of Withholding $30 Million In No Surprises Act Independent Dispute Resolution Awards</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Anthem has been accused of improperly withholding $30 million in independent dispute resolution awards owed to healthcare providers under the No Surprises Act. This dispute matters because delayed or withheld payments disrupt provider networks and increase administrative friction within commercial healthcare markets. For self-funded employers and benefits managers, payer disputes surrounding out-of-network claims threaten to drive up operational costs and strain provider relationships, ultimately impacting overall healthcare cost management strategies.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BenefitsPRO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 15:50:33 GMT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPZVY4WmI4LTBCSEEwZHhsVnd6dUl2MzJvRUs1RUc3TDkzZ2xFTXRJdXV1Sk4ybDA5NXJ4eDhxdjF1X2hoOGxpQXdvUTRMMkhuWGxTNWNVOUYtZXE0Q2VFamFsSXo4Q2ZlT2tNLXQzTXRGdFRuVTlBNXhRRTUyVDBNUzcxTEdpTjhzOTNFTlN0MTkyOTNMaW9jSzZ0NUlBLVNvbFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rising Healthcare And Pharmacy Costs Threaten Small Business Sustainability</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Escalating healthcare costs are placing an unsustainable financial burden on small and mid-sized businesses, threatening their operational survival and forcing employers to reconsider how they sponsor health coverage. This trend matters because self-funded and fully insured employers urgently need innovative cost-containment strategies to manage medical and prescription drug inflation without compromising talent retention. For PBM partners and employee benefit providers, this creates a critical opportunity to deliver transparent, flexible pharmacy management solutions that help smaller employers mitigate runaway healthcare spending.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Washington Times</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 19:54:55 GMT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPaEhkZTZ1cnE2RF83WUs2dkNKZmw2N1p6YVU5VHVYWW4yYUZrVUJ4eTM2a2xjUkdULS1TZHVYOC1MM2s2QlZ2OGp0VXd1YTI4RkdjUDhucmNRckVVWnNQYTJBTDIycFFJX3NkX09wYkVHaHpRMUNtUGUzSjVfZjQ1TGdjUjhnNWFKYjMzTC04VG1jbC1xcnlpcXpuWkd2dmM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hidden Market Dynamics Drive Up Healthcare and Patient Costs Significantly</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Investigative reporting highlights how opaque market forces and pricing structures continue to add thousands of dollars in unexpected healthcare expenses for everyday patients. This trend underscores the persistent challenge of healthcare affordability and cost transparency within the commercial insurance space. For self-funded employers and benefit managers, these rising underlying costs emphasize the urgent need for proactive pharmacy and healthcare benefit optimization to protect plan members from escalating financial burdens.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KFF Health News</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 09:48:23 GMT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNdWtqcVp4b2ZlWE1Sdk5mcEF2bU1oazVIM2JmQjNmSjNiR2hoWXcwd3Fod0VQbktsUjk1Q2R1T0FfUHpvdzZyS0tfczlyeGR5QzhzSUsxZFl5N0FpekI0UHpnSWJFQy1BWWNJYTg0ZmY1SjduSWpsNzFKRnBlR1QyakxKV0t4UDZTRkdMMGZqTVlVaXBSYTRFUnRCb0k0TG8yZTctbWg3bVpveEwyOElR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sandoz Expands Focus on Biosimilars to Drive Market Growth</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sandoz is strategically increasing its focus on expanding the biosimilars market to offer lower-cost alternatives to traditional biologic treatments. This initiative matters to self-funded employers and benefit managers because wider adoption of biosimilars can significantly reduce specialty drug spend and overall healthcare costs. Key business implications include heightened competition among manufacturers, which is expected to drive down prices and create new opportunities for pharmacy benefit managers to optimize plan formularies.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Drug Store News</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 13:38:48 GMT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9FTkczVUFQaTc2WTR2T3dlcFlpTzhYSk1vcFcxcVpJaWVPMlpQaGdBcUlPajFscE1ReF9XX0U0YVhVQUxaOUx6Z1p6THVRc3RxUWhqOE42TUNLQ2tZZDVWLUpqX3VZVnpsb2pTTzBFSWE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Forus Secures $150M Series C Funding To Expand AI-Powered Medication Access Platform</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Forus has successfully raised $150 million in Series C funding to scale its artificial intelligence-driven platform designed to streamline medication access. This development matters to self-funded employers and pharmacy benefit managers as technological innovations increasingly target administrative friction and affordability in prescription drug delivery. The expansion highlights growing investor confidence in digital health tools that could reshape how specialty and traditional medications are sourced and managed for employee benefit plans.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Fierce Healthcare</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 18:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPNE5sSDQzWV8tcUJ0Ym44cENnVF9fbWxiWEg5Ni1Xb0dlOFBvSE83TTd4YnFiRWlMUEFLekZtSl9mRE1rcU9jU3puaWF3cmRrSXF5QVB5VTVBb2J0Z3hzSHlQaWwyM2h5WC11ZlJGb2ZaZnktSVBILXBzaVM1VVUwZm9UdjJTZF9ocnh6X0tn?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Supplemental Health Benefits Drive Higher Rates Of Employee Retention</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>A recent industry report highlights that offering supplemental health benefits significantly improves employee retention for self-funded organizations. This matters because employers are increasingly seeking holistic benefit strategies to combat turnover and manage overall workforce expenses in a competitive labor market. For businesses managing employee benefits, integrating supplemental coverage serves as a valuable tool to enhance total compensation packages while supporting long-term workforce stability.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BenefitsPRO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 21:26:31 GMT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPaDdVeWJKeXdjRkZEWGgwQTFzWEFYeGZsTUxtVUx2ODM4S3VZQ0pZUFJGNU1JektEeUlOVVJwcVNGaVUyTkRtS19qVmVzaEJ5M1o4QVdCVi13NzcwUmNaRi1lTVRfaWJzQjhsYXFYNnNRVW9tSDdWUl9aeEp5djVGNDIzZjMtZWVGRTdKeDN5RTZuc3ZBLWlnLQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Surging Medical Costs Compress Health Insurance Profits And Threaten Employer Plans</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Major health insurers are experiencing declining profits as surging medical and pharmaceutical costs outpace premium growth. This trend matters because sustained financial pressure on carriers often trickles down to self-funded employers through higher stop-loss insurance rates and increased administrative fees. Consequently, employers must aggressively adopt advanced cost-containment strategies, such as tighter PBM oversight and specialty drug management, to protect their self-funded health plans from compounding market inflation.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BenefitsPRO</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 18:09:25 GMT</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNbTZ1VWJrU3RZNGhhZlZpV05hZkNKVG9zbF9IcHhnZlpBb3REMm0xZURuWlczaXBaTW9zb0lhMG16QVp3YTBGdE5TVlMtbFhVejdiUVFTSC1lUlhTMmxXU2tRNGlGUlRLU1hMTjZiV2RkTlRQczExU3RmOGkzZGdtUWFJQjJBNjZBR1Z3eWJ3TF9PVTFqU1BvTjlPbW1WZw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Anthem Accused of Withholding Millions in No Surprises Act Independent Dispute Resolution Awards</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Anthem is facing allegations of unlawfully withholding approximately $30 million in independent dispute resolution awards owed to healthcare providers under the No Surprises Act. This matter matters because payment delays and compliance friction within dispute resolution frameworks directly impact healthcare provider relations and broader cost-management dynamics within commercial health plans. For self-funded employers and benefit managers, ongoing friction in dispute resolution processes highlights the continued volatility of out-of-network claims processing and underscores the need for vigilant oversight of payer administrative practices.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BenefitsPRO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 15:50:33 GMT</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPZVY4WmI4LTBCSEEwZHhsVnd6dUl2MzJvRUs1RUc3TDkzZ2xFTXRJdXV1Sk4ybDA5NXJ4eDhxdjF1X2hoOGxpQXdvUTRMMkhuWGxTNWNVOUYtZXE0Q2VFamFsSXo4Q2ZlT2tNLXQzTXRGdFRuVTlBNXhRRTUyVDBNUzcxTEdpTjhzOTNFTlN0MTkyOTNMaW9jSzZ0NUlBLVNvbFE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Modular Medical Secures National PBM Contract To Expand Tubeless Insulin Pump Access</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Modular Medical has signed a distribution agreement with a major U.S. pharmacy benefit manager to provide commercial access to its Pivot tubeless insulin patch pump. This development matters because it integrates innovative diabetes technology directly into mainstream pharmacy benefit channels, potentially improving patient adherence and outcomes. For self-funded employers and PBMs, this partnership signals a growing trend toward incorporating advanced medical devices into pharmacy benefit management, which could impact specialty drug and device cost-management strategies.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>accessnewswire.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 17:55:42 GMT</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxOUHRkc3dGZUt2RzBpckI2b0JiZnNIV2Q3d0s2MzJhOGI3YVJYR0NzemliVldwdEpZSWpNZzR0Y2oxSTBxbmF5NXUycmZrS0hDZGRScVVRUHh5djhSX3E5UjFnZmd5SFk5bkJjb2hhMkhSRjBOcUY0aEFwUVROS3lja0k4emxfME9VOEF2dFFlVEFoalVyUl9FRUhzZVBwc0Jtb2xaUlNlelpPMWdMamoxM1BGMGE4ekFzV2FJeFplMmp0Z3ZyUFNXTUhBX0hOeVZEQVFQTUFsYktqQ2RLaTBjbURTT0U?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>New Kansas Law Drives Significant Cost Savings Through Pharmacy Benefit Transparency</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kansas has enacted legislation aimed at increasing transparency within pharmacy benefit management, which a local pharmacist projects will save the state millions of dollars. This regulatory shift matters because enhanced oversight of PBM practices directly impacts drug pricing transparency and overall healthcare expenditures for self-funded and state-level plans. For businesses and benefit managers, this trend signals a broader movement toward stricter state-level PBM regulation, offering potential opportunities to curb rising prescription drug costs and demand greater accountability in pricing structures.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Wichita Eagle</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 09:36:00 GMT</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBJVjNMemRnaU8zUlBIWTc4aXdmQ2p5dmpGQkhJbmEtV1FEYWhZWGx5eDFjRENzZjgtdVBDNk1kQ2dkZzhVQUJCY0NGZFZwYXY3QjdpMC1oUTgzdGVRMk96R2FrTnJvSnRfUy05b3EwUWFGQ25PNGNZRdIBeEFVX3lxTE01SkNnVkR2NUJJc196WXdvR3QyX1I4MDRXRG9rdGdrYmFuSHJBdEMzOEJBV3llQ2hSUU1oRnJSUHJSYU5LUGR1WjF1ckxMekJreGtsaTBCdTFXNndoTXN2bmNZMzE5aHA2djJCSXA0dmF4RG50cUI4Vw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Benefits Brokers Must Adapt Strategies To Combat Rising Employer Health Care Costs</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>As soaring healthcare expenditures continue to strain self-funded employers, industry experts are urging benefits brokers to abandon traditional advisory models in favor of more innovative cost-containment strategies. This shift is critical because employers are increasingly demanding proactive solutions to manage soaring specialty drug and pharmacy benefit expenses. For organizations like RxBenefits, this evolution highlights a prime opportunity to partner with forward-thinking brokers who can deliver data-driven pharmacy benefit optimization to control plan costs.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Insurance Business</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Wed, 09 Sep 2026 01:28:45 GMT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPbWo1WVBBY01CSkpGdXkzUEUweHFxcnRkaVQxOC1rWGJDSVpzNUVFWkFQdzNrRmJOQV9PdVM2OE9DYVlpcVB5bEh2MV9UeEtVaTdNcGFmeERBMjJNT2VMZkxFSVFCU0xjZlpNS1NITDRwcjdyRFRtUk9jMVpFNTgtX0x6QlRFTkhhelRZWkZiNjBpbW5JME5aTWpseU0zMldPcU9xQmk2UnQ0RG5VUms2NUNhY0RJYW5GbkxVYnB4UV8tOFI5Smd5WW1B?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Employers Health and Judi Health Partner to Launch Modular PBM Solution StarkRx</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Employers Health and Judi Health have collaborated to introduce StarkRx, a new modular pharmacy benefit management (PBM) solution designed to give self-funded employers greater flexibility and control over their pharmacy plans. This partnership matters because it addresses growing employer demand for transparent, unbundled PBM services to combat rising drug costs. For the broader industry, this signals a continued market shift toward modular benefit architectures, allowing plan sponsors to customize services and optimize cost management without relying on traditional, monolithic PBM contracts.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>IndyStar</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 15:28:37 GMT</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOSGVsOEZDSmo5N2gxZXRzTnhjbWhPNGhaNktLRHZjUDFRWGFRWEJ1N0RvNGc4QnN6WUk3aHBaUXRBdkkzeFgxWW1YankxSWdXS3BxcnhhZ2tzelctM0h2TzN6RlFjaEVlVXlBX2ZpN2c1aVltOFpOSTFQbDEzOG42ZlZ0WU1fUEpBUFBDa2g0ZXJiQVRMc2JKaXUyZ1FvNG40MTVEYjF6dGlOZFVpVkJULUFBN1Z0bTND?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>The Impact Of Health Reimbursement Arrangements On Broker Roles In GLP-1 Coverage</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>The rising utilization of Health Reimbursement Arrangements (HRAs) is sparking concern over whether traditional insurance brokers will be bypassed in managing high-cost GLP-1 weight-loss medications for employers. This trend matters because it shifts benefit-steering mechanisms and alters how self-funded employers design and finance their pharmacy benefit offerings. Consequently, stakeholders must monitor these evolving financing structures to protect advisory relationships and navigate escalating specialty drug expenditures effectively.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Insurance Business</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 18:52:24 GMT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQOS0yc3I2cWp2MEUyWmlOZzhDRWsya2F1YlFlT3MxQ01HS0hXXzEydTYxZnZsalpxSXp4dEx1d3E2SWRQQ3Z6Nks0ckl0eWwySXBQRHMtRUI2eHlTeGNsaERIeURKbUsxN29VcEEwSDkxU0tBSDlxSDd5ektfLTlEQVBFZy1JR0ZvQ28ybXRMdTFUR2RORXVzYko3aTRGVG9WdFBIX3J1LVVHWDRzX2t2Wm4xTnd6c1NWanRmeA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Employers Health and Judi Health Partner to Launch StarkRx Modular PBM Solution</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Employers Health has teamed up with Judi Health to introduce StarkRx, a new modular pharmacy benefit management (PBM) solution designed to give self-funded employers greater flexibility and control over their plan designs. This partnership matters because it addresses growing employer demand for transparent, unbundled PBM services that can be customized to combat rising specialty drug costs. For the broader market, this signals an ongoing shift toward modular healthcare solutions, threatening traditional PBM models and creating new competitive dynamics in self-funded employee benefits management.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Knoxville News Sentinel</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 15:41:42 GMT</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOTGphd0xkSlA5dFFMLWhIU0ZMUjVncWY0T2FTRllpM1MwMEwxWFRFc2FkQ1RTWmRDS2RyT0ZTalVyMjhwLWJUdTlUOGJXTGhnaTVPNzRUSl9rNUZTTmtHWi1fOFZ4Wmc5OF8zMFJwOGp2TXA4dmlOcGZmRUFGVzI3SEJ0ZE5MSWkxd1N0aTBOelcwNjNsZHRnNFZFUFJack8ySEpNb0hVdWpvbUJQQTdkaDhudTJiRUxE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Benefits Brokers Must Adopt New Strategies To Manage Rising Employer Healthcare Costs</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Industry discussions highlight that traditional approaches to managing employer-sponsored health plans are no longer sufficient amid escalating medical and pharmaceutical expenses. This shift matters because self-funded employers increasingly rely on brokers to deliver innovative cost-containment solutions beyond standard renewals. For RxBenefits and channel partners, this creates an opportunity to position pharmacy benefit optimization as a critical component of the modern broker playbook.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Insurance Business</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Wed, 09 Sep 2026 01:28:45 GMT</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPbWo1WVBBY01CSkpGdXkzUEUweHFxcnRkaVQxOC1rWGJDSVpzNUVFWkFQdzNrRmJOQV9PdVM2OE9DYVlpcVB5bEh2MV9UeEtVaTdNcGFmeERBMjJNT2VMZkxFSVFCU0xjZlpNS1NITDRwcjdyRFRtUk9jMVpFNTgtX0x6QlRFTkhhelRZWkZiNjBpbW5JME5aTWpseU0zMldPcU9xQmk2UnQ0RG5VUms2NUNhY0RJYW5GbkxVYnB4UV8tOFI5Smd5WW1B?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Four Independent Pharmacies Permanently Close Across Michigan Amid Rising Operational Pressures</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Four independent pharmacies in Michigan have announced permanent closures, reducing local healthcare access points for patients. This trend reflects ongoing financial pressures on community pharmacies, which struggle with squeezed profit margins and reimbursement challenges. For self-funded employers and pharmacy benefits managers, such closures threaten network adequacy and could drive members toward higher-cost retail or mail-order alternatives, impacting overall plan utilization and costs.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>wcmu.org</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 19:50:00 GMT</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPd196RnFtM1BDTVN0VEZzcDhoSTRMMUxGSFVlcFZXVmY3d2hIUUQteGJ6cFpaYkN6Q3JCQUdkeUM2WlhfQTF3TjJIQ3RLUzBZTTQzSTkxWTU0TWZYV0JqMC1BSjhmYnpNem5YTFRxd01vaTBCS0lhT3htcl9JTWNXLTdqT2tNNjZKaGRrMEF5R1lfeHlHaVBWRGdER3laTktjVmRBWFZLNGMzYU9LWWk1OXQ0N2x2T1FySklsc2EzNA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Modular Medical Secures National PBM Contract To Expand Tubeless Patch Pump Access</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Modular Medical has signed a distribution contract with a major national U.S. pharmacy benefit manager to broaden patient access to its Pivot tubeless patch pump for diabetes management. This partnership is significant as it integrates innovative diabetes technology directly into mainstream pharmacy benefit channels, potentially increasing utilization and influencing device coverage trends. For self-funded employers and benefit managers, this signals a growing emphasis on incorporating advanced medical devices into pharmacy benefit frameworks, which may impact overall plan design, member cost-sharing, and specialty diabetes management strategies.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>accessnewswire.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 17:55:42 GMT</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxOUHRkc3dGZUt2RzBpckI2b0JiZnNIV2Q3d0s2MzJhOGI3YVJYR0NzemliVldwdEpZSWpNZzR0Y2oxSTBxbmF5NXUycmZrS0hDZGRScVVRUHh5djhSX3E5UjFnZmd5SFk5bkJjb2hhMkhSRjBOcUY0aEFwUVROS3lja0k4emxfME9VOEF2dFFlVEFoalVyUl9FRUhzZVBwc0Jtb2xaUlNlelpPMWdMamoxM1BGMGE4ekFzV2FJeFplMmp0Z3ZyUFNXTUhBX0hOeVZEQVFQTUFsYktqQ2RLaTBjbURTT0U?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Kansas Lawmaker And Pharmacist Anticipate Millions In State Savings From New PBM Transparency Regulations</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A new state law in Kansas introduces stricter transparency mandates for pharmacy benefit managers (PBMs), which local healthcare experts project will save the state millions of dollars. This matters because it highlights the growing legislative momentum at the state level to curb hidden PBM costs and reallocate drug spending. For self-funded employers and benefit managers, this trend signals increased regulatory scrutiny on PBM practices and opens potential pathways for greater cost containment and pricing visibility in commercial health plans.</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Wichita Eagle</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 09:36:00 GMT</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBJVjNMemRnaU8zUlBIWTc4aXdmQ2p5dmpGQkhJbmEtV1FEYWhZWGx5eDFjRENzZjgtdVBDNk1kQ2dkZzhVQUJCY0NGZFZwYXY3QjdpMC1oUTgzdGVRMk96R2FrTnJvSnRfUy05b3EwUWFGQ25PNGNZRdIBeEFVX3lxTE01SkNnVkR2NUJJc196WXdvR3QyX1I4MDRXRG9rdGdrYmFuSHJBdEMzOEJBV3llQ2hSUU1oRnJSUHJSYU5LUGR1WjF1ckxMekJreGtsaTBCdTFXNndoTXN2bmNZMzE5aHA2djJCSXA0dmF4RG50cUI4Vw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Employers Health and Judi Health Partner to Launch StarkRx Modular PBM Solution</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Employers Health and Judi Health have joined forces to introduce StarkRx, a new modular pharmacy benefit management (PBM) solution designed to give self-funded employers greater transparency and flexibility. This partnership matters because it addresses growing employer demand for unbundled, customizable PBM services to better control escalating healthcare costs. For the broader market, this signals a shift toward modular vendor arrangements, allowing self-funded plans to bypass traditional opaque models and optimize specific components of their pharmacy benefits.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>IndyStar</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 15:28:37 GMT</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOSGVsOEZDSmo5N2gxZXRzTnhjbWhPNGhaNktLRHZjUDFRWGFRWEJ1N0RvNGc4QnN6WUk3aHBaUXRBdkkzeFgxWW1YankxSWdXS3BxcnhhZ2tzelctM0h2TzN6RlFjaEVlVXlBX2ZpN2c1aVltOFpOSTFQbDEzOG42ZlZ0WU1fUEpBUFBDa2g0ZXJiQVRMc2JKaXUyZ1FvNG40MTVEYjF6dGlOZFVpVkJULUFBN1Z0bTND?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Unseen Market Dynamics Driving Up Out-of-Pocket Healthcare Costs for Patients</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Recent investigative reporting highlights how complex, hidden market forces within the healthcare and pharmaceutical supply chain are inflating patient out-of-pocket expenses by thousands of dollars. This issue directly impacts self-funded employers and benefits managers striving to control rising healthcare expenditures and protect plan members from unexpected financial burdens. For organizations like RxBenefits, this underscores the critical need for transparent pharmacy benefit management strategies and proactive cost-containment solutions to shield employers and employees from escalating drug and medical costs.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KFF Health News</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 09:48:23 GMT</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNdWtqcVp4b2ZlWE1Sdk5mcEF2bU1oazVIM2JmQjNmSjNiR2hoWXcwd3Fod0VQbktsUjk1Q2R1T0FfUHpvdzZyS0tfczlyeGR5QzhzSUsxZFl5N0FpekI0UHpnSWJFQy1BWWNJYTg0ZmY1SjduSWpsNzFKRnBlR1QyakxKV0t4UDZTRkdMMGZqTVlVaXBSYTRFUnRCb0k0TG8yZTctbWg3bVpveEwyOElR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Employers Health and Judi Health Partner to Launch Modular PBM Solution StarkRx</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Employers Health and Judi Health have collaborated to introduce StarkRx, a new modular pharmacy benefit management (PBM) solution designed to give self-funded employers greater flexibility and control over their pharmacy plans. This partnership matters because it addresses growing employer demand for transparent, unbundled PBM services that combat rising drug costs. For the broader industry, the launch signals an accelerated market shift toward modular benefit architectures, pressuring traditional PBMs to offer more transparent and customizable contracting models.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>IndyStar</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 15:28:37 GMT</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOSGVsOEZDSmo5N2gxZXRzTnhjbWhPNGhaNktLRHZjUDFRWGFRWEJ1N0RvNGc4QnN6WUk3aHBaUXRBdkkzeFgxWW1YankxSWdXS3BxcnhhZ2tzelctM0h2TzN6RlFjaEVlVXlBX2ZpN2c1aVltOFpOSTFQbDEzOG42ZlZ0WU1fUEpBUFBDa2g0ZXJiQVRMc2JKaXUyZ1FvNG40MTVEYjF6dGlOZFVpVkJULUFBN1Z0bTND?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Shifting Drug Pricing Policies Force Major Overhaul in Commercialization Strategies</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Recent sweeping drug pricing policy reforms are causing pharmaceutical companies to fundamentally restructure their global commercialization and launch strategies. This shift matters because regulatory and pricing pressures directly influence drug development pipelines, market availability, and long-term cost trajectories for prescription medications. For self-funded employers and pharmacy benefit managers, these evolving market dynamics signal potential changes in future drug pipelines and cost-management approaches for specialty therapeutics.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fierce Pharma</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Wed, 09 Sep 2026 04:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOQVh0bmsxYmFQY3ZDNzZKR3UydVFSUlpBQ2I5NFRDOVMzMEZFVVpaVEZFSHNXS1ZjY2p4akxyc20tUWUyVURpMVBRSzR0MGZuVE9mc01ZUXptYWlIYUg5QjdRVjN5ZzBULVRqQ1lHN2wxOEdad0RZTC14dnFTbHdSazJKbzNEOW45bHJJM2NkZ2xHd3R2U01ZaEdsRmN6R2doZ3RON1hNSzZwcXNKOU9VS21lY1BIRW5oLTdmMDMyMXM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>The U.S. Drug Pricing Paradox and Its Impact on Commercial Healthcare Costs</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Forbes examines the complex U.S. drug pricing landscape through the launch of RevMed’s new therapy, Rasonque, highlighting the ongoing tension between pharmaceutical innovation and affordability. This pricing paradox matters greatly to self-funded employers who bear the brunt of escalating specialty drug costs without public sector price controls. Consequently, plan sponsors must adopt proactive pharmacy benefit strategies and robust cost-containment measures to manage high-cost specialty introductions effectively.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 13:15:24 GMT</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOcGgxVDBzclBpNVpqRU1kMjNXS1Vkd0pWWUN5dW5ORlFlMjdXUnZmaDVNWWwteW84bS1zaUtaQ3FoQ0staGZaWndDSWVCRzE0NDlTcmd0cFNBQVc0SjI2X2YzOUlkdzVqdDZiUl9iblNQTEcxSUs1MUFna1E5N2JsMjNXcDZacG0wd1lpWW8tYXhVVzZJZFBZYl9OeERMOW56RE8tWjNicnZFeU5IQXlJUTJOXzl5RllrZVZCSWNR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of GLP-1 Pricing and Program Terms Between PlexusDx and Calibrate for 2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PlexusDx released a comparative market analysis examining the 2026 pricing structures and program terms for GLP-1 weight-loss treatments offered by competitor Calibrate. This evaluation matters to self-funded employers and PBMs because navigating escalating anti-obesity medication costs remains a primary healthcare budget challenge. For the business, understanding competitor program terms and pricing transparency benchmarks helps organizations better advise clients on optimizing specialty drug management and containing long-term plan expenditures.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PlexusDx</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 19:11:45 GMT</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNZm8weENjNFAxNmJJbldZUTdCYzNzb1hwdUVObWJjMlBHVDRtS24zcUxjRTNHXzVkWFFHM3VjcnJJeWVycTFGQThpVG9jZzg4UTlRR2I2QnkyLVloQlh3YTd2aHlIakEwTEUxRldnS2RCMXU0SWFvb3drX28zSTBubTM4WmxheThEMFhHVzhSVFF1V3hSVXJyWS1NMzZDYUtVM05rQ25wbw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Improving Employee Benefits Literacy to Drive Healthcare Value and Utilization</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>A recent industry report highlights that enhancing employee understanding of their health benefits is a critical frontier for maximizing the return on investment for self-funded employers. This matters because low benefits literacy often leads to underutilization of cost-saving programs and poor healthcare decision-making among employees. For pharmacy benefits managers and employers, investing in education strategies helps employees navigate complex drug and health offerings, ultimately mitigating avoidable medical and pharmacy costs.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Insurance Business</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Wed, 09 Sep 2026 01:28:45 GMT</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQcEpsS2RVUXZ0Q21wRmdaSFZ0QThZSU9pNFNETXpZbGRSenlWSmd4cVhMTDMxSmZFV3h5eFVPT21nR0VlVVdTa3I4SlVlZzVQaHQ2QThlTzVZcjJKM0FBUExHNTFhWUI5VWNCX2pvWTRGUEZ2cms1a0cyWFl2aEVTNmF0S21pNTFrZTg1ZHJoZDJwZ2ExcTl5bm1uQlFXbVZETlFneV9iWlBzSVNQOGY1aUpHUnBiSGxFam1hd29scw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Employee Pushback Intensifies Following Major Payer Decisions to Drop GLP-1 Coverage</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Employees at a major organization launched a petition after Cigna eliminated coverage for weight-loss medications, highlighting the growing workforce friction around cost-containment strategies. This backlash matters because it underscores the intense employee demand for anti-obesity drugs despite skyrocketing plan sponsor expenses. For self-funded employers, this event signals that restricting high-cost specialty benefits requires careful change management and communication to prevent severe employee dissatisfaction and retention challenges.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>HR Executive</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 12:00:33 GMT</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOOEtHd2lqaTBtcTVhMHRsTTkyQXdXM050VVRackpBVjFrNVl3SFVoUGN1NXo4T2dxZTMwdzJsY3FlLUxxbEpDeUJpcEtuX3dUXy1IQVJ0Z2ZVWGV6bkFNZWU3ZDlLZlVwU3RKQ2VrSWo1elY2RmEyaHJ2cHZQeUdMWlBuVnJKLXpJTlJYbjdDY0NPQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Projected 8.2% Spike in Employer Health Care Costs Demands New Cost-Management Strategies</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Recent industry projections indicate that employer-sponsored health care costs are set to surge by 8.2%, driven largely by escalating medical and pharmacy expenses. This sharp increase poses a significant financial threat to self-funded employers who are already struggling to maintain affordable comprehensive benefits for their workforces. Consequently, organizations must urgently adopt advanced pharmacy benefit management solutions and targeted cost-containment strategies to protect their bottom lines while sustaining employee health coverage.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Word &amp; Brown General Agency</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 20:31:00 GMT</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOUTZfNDN5UmlUdXo0NS1lZU05T0QxbzM4d0dDZHlpVktIaGNybWZWUVg4NlFHVFRTbEw2M2ZSbEMxOHg4QmFja250RGdhcnZ1VzNfY2xlRHA4ay1WeWxhbEVxTEJEYUUwdlhmSW9Hc1h4alRnNW5HMUxfYko3RnhPQkw5WTVmTERRZ0hPbnh3?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Department Of Labor Releases Strict Enforcement Guidance For Mental Health Parity Compliance</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>The Department of Labor has issued new enforcement guidance regarding mental health parity requirements, setting stricter compliance standards for employer-sponsored health plans. This matters because self-funded employers face heightened regulatory scrutiny and potential liability if their group health plans—including pharmacy and medical benefits—fail to provide equivalent coverage for mental health and substance use disorders. Key business implications include the urgent need for plan sponsors to audit their benefit designs, pharmacy utilization management rules, and prior authorization criteria to ensure full compliance and mitigate costly legal risks.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Law360</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 21:59:00 GMT</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE9WQ0JvM2NncXlHbTcyMjRLdzhuOTBhY1Q4QXVJR2NzRzBRcUtIdU5vbTdzRHFaUjM1M1BwbUVSUW80cjFOM1NVXzJTTUxPdnJxNlhmbHNB0gFWQVVfeXFMT1ZDQm8zY2dxeUdtNzIyNEt3OG45MGFjVDhBdUlHY3NHMFFxS0h1Tm9tN3NEcVpSMzUzUHBtRVJRbzRyMU4zU1VfMlNNTE92cnE2WGZsc0E?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>No Surprises Act Independent Dispute Resolution Costs Surge to $22.4 Billion Amid Rising Billing Disputes</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Independent dispute resolution costs under the No Surprises Act have climbed to $22.4 billion as healthcare billing disputes between providers and payers surge nationwide. This massive financial accumulation matters because administrative and arbitration expenses continue to inflate overall healthcare delivery and operational overhead. For self-funded employers and benefit managers, this trend signals ongoing friction in healthcare pricing transparency, potentially leading to higher indirect costs and heightened pressure to secure predictable out-of-network reimbursement strategies.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>insurancenewsnet.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 16:11:22 GMT</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPMjIzZGdzYXNsYlpJWVdXLVZHWGZ0TDhNdUJxMXdtWVlWeG5DaTk5dW5zemFENk41ZXFzanFJbW9JNHZKOWhkeDZKaGZJM0J2amFfclNDUGU2MHVodUREUlhTOTZqNXRoSS13WGR1TG1NUm5oSnZ4YzhFU2did19iano1UV91V3RHVENSdzRjN01EREVwcnQtQWhnWjJYcHhYdTZWZWJocHZUX3JNbjUzWA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Rising Healthcare Costs Drive US Small Businesses to Drop Employee Health Insurance Coverage</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Surging healthcare expenses are forcing a growing number of small businesses to eliminate health insurance benefits entirely to stay financially viable. This trend matters because it shrinks the traditional employer-sponsored insurance market, leaving employees without coverage and shifting more financial risk onto individuals. For self-funded pharmacy benefit models, this highlights an urgent market demand for innovative, cost-containment strategies that help smaller employers maintain affordable benefits without pricing them out of the market.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Heartlander News</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 21:21:14 GMT</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNTDBKLXdsdjByNzFqZWVSZWI1T0twaGdfdDQxTFlzemY3X01ueVhLUkFUUDV4ZFpfU29YSkx4TTFnZnRUOTVxeTMySHlXeU1rTDUwSEk5QUFSNlZSWXJ2b2R0NkgyT0RCWGhEYS1rbWQzcDNpS0VsUmtfYUpuMjM0M3F4NzkwOE8zRTFqMk10aHRrNWF2VWY5UTJFMW9mWmlockNKMWd6MEhBcmJZLUhOejE0dS12YWs?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>The US Biosimilars Market Projects Rapid Growth Driven by Specialty Drug Adoption</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>The US biosimilars market is projected to nearly double in value, fueled by increased adoption across key therapeutic categories and shifting payer strategies. This growth matters because lower-cost biosimilar alternatives offer self-funded employers significant savings opportunities to offset rising specialty drug expenditures. For benefit plan sponsors and PBMs, this trend underscores the necessity of aggressively integrating biosimilars into formularies to effectively manage healthcare costs and curb trend inflation.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Managed Healthcare Executive</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 22:07:23 GMT</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPS3NfYU10Y0NLY0hhTzBka2cxM2NXZ0hEWHFxQ2x1WS1NcVJNc2Izc3ZiMGVTOTlhd29sVWoyMl9JbzRuZVl0amZ5QlFKc3pGQ1Y0Y3h4Y3dIUG1aekNDT3pfaTBoaDU3NElHXzB2QUgyX3ctYmVCQnVRSlRoTk5wMF9ILUhSYThTeTFncmgzbzNFXzFCQlhfUi12dE9kVk9lU29qNjgwOWpEeUQyNkNVaFRtTUVhRE9aZkpaT0oxTXpMYkJYc293aVZQaU1EYXM0eTl6OXNB?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sandoz Launches Ambitious Long-Term Strategy to Develop 100 Biosimilars Backed by $300 Million Manufacturing Investment</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sandoz has unveiled a strategic growth plan aiming to bring 100 biosimilar products to market by 2040, supported by a significant $300 million investment in a new manufacturing facility. This expansion in the biosimilars market matters because it promises to dramatically increase competition for costly biologic therapies, driving down drug spending for self-funded employers. For business operations, this robust pipeline signals greater market availability of lower-cost alternatives, creating essential opportunities for pharmacy benefit managers and plan sponsors to reduce specialty drug expenditures.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Fierce Pharma</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 18:45:54 GMT</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPdjBHbU9uT1pER0gteUhnVzc1RkpwWlAzQVFHWk11QmktQkdkLTkydjdPSEJSS014RlVRSDUzNHpjNXEtWXppZF96MDBXNXNKQXVYWW1XQ2c4VG5fSWZVWGF2Q1BIUEFiZ0ZiMGxQV1FtNUl0VE15OUV2RkRiVkVwWU1lQmdOVHBsbnJKTEZQbDNEVmt6NlJKUHJibUxjZmp3OEtqT1FIU3BBcE9pX20xekd2RC1VMnVULTNEYg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sandoz Expands Biosimilar Portfolio with Ambitious Growth Target by 2035</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sandoz has announced a major strategic push into the biosimilars market, setting a goal to double its overall group sales over the next decade. This expansion is significant for self-funded employers and pharmacy benefits managers as increased market competition from alternative biologic treatments helps drive down escalating specialty drug costs. For RxBenefits and its clients, the growth of the biosimilars sector unlocks valuable opportunities to curb runaway healthcare expenditures and deliver more affordable alternatives to expensive reference biologics.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>WTVB</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 11:01:36 GMT</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPQzZzMW5lTGNkdEtjT3J1R1hHWTcwUEdpYVJ0QVRqNV9MLWZObHdBMnNYRlJoVDZlSFprZ1RiXzNNSnhqa1o2LVZjajRiMTR6SzBqYURPZXhpVENLcGJTZEF2ZGVVRmRQWGJ5RE5NYmFiMXN0bEtRSFR0TXN1Q0JPQ21makx3TWZvbGVLTHJ6YlhDTUdoZm9RRnAyX0hwUzQ5cGdQcg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sandoz Expands Focus on Biosimilars to Drive Market Growth</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sandoz is strategically increasing its focus on expanding its biosimilars portfolio to capitalize on shifting market demands. This matters because wider adoption of biosimilars is critical for self-funded employers and pharmacy benefit managers seeking to lower soaring prescription drug expenditures. Key business implications include heightened competition among manufacturers, which is expected to create significant opportunities to reduce specialty drug costs and deliver greater long-term savings for self-funded health plans.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Drug Store News</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 13:38:48 GMT</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9FTkczVUFQaTc2WTR2T3dlcFlpTzhYSk1vcFcxcVpJaWVPMlpQaGdBcUlPajFscE1ReF9XX0U0YVhVQUxaOUx6Z1p6THVRc3RxUWhqOE42TUNLQ2tZZDVWLUpqX3VZVnpsb2pTTzBFSWE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sandoz Launches Bio 100 Strategy to Deliver Over 100 Biosimilars by 2040</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sandoz has unveiled its ambitious "Bio 100" initiative aimed at bringing more than 100 biosimilar products to market by 2040, a move projected to double its net sales and expand profit margins. This aggressive pipeline expansion matters significantly to self-funded employers and pharmacy benefits managers because the rapid proliferation of biosimilars is expected to drastically increase market competition and lower specialty drug costs. For employee benefit managers, this trend creates substantial opportunities to drive long-term healthcare cost containment by shifting utilization toward more affordable biologic alternatives.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TradingView</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 22:11:12 GMT</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxOc2dHWEpQWUNPN0JEZWFvVWI5eHE2Y0JuNnVXbGt3SHRER3NkMXkta2FTRWROLTBYUEk3cnpyYzg4QzVtQ21lVGhfOEg5cmhlRTVYUzdMM2hVdGNmbzZyZ2xneVFQU2dKVEFqa1F4THNwVGdKdlFpVGI4a2RuTVZWaC1hSkgxVXZjTXRfbUcyLW1GeFNrNHdUS3FCdXJJakotY04zN3NuMzBCSWd1dUNKOFRuU1lReEZBSDhPZElZWVFJbUxTX3NOY3gzMk1KMGxIWXZMT1d0R2xncUZMTDVMM1g1dElsRGVKZlFkT1dXMnM4TkdJdmRkUDVPRjRDbW8xeE1rVnc1bmw1WmZXcWc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandoz Stock Rises as Biosimilar Pipeline Drives Long-Term Growth Strategy</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandoz shares increased by 5% following the announcement of an ambitious 2035 growth target fueled heavily by its expanding biosimilars portfolio. This matters because the accelerated adoption and market entry of biosimilars represent a primary mechanism for self-funded employers and pharmacy benefit managers to reduce specialty drug spending. For the industry, this signals a maturing market where increased competition from lower-cost biologic alternatives will significantly alter drug pricing dynamics and formulary management strategies.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Investing.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 10:36:34 GMT</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxObXBrbjB4bHJsSjJteTY2YkxhSEtFSkxaQy1udVF0ZnJTaEZfcjlRSEhLZ0ZtUnpzZndtWTYwdE51TTZ4OHBVQTh5RTBjRzdLbmM4QWhOblFtN3VfcjlDV2JES3hPLWhaOG1nNHdSUG01TkFXV3kwa0JTblpyR3NfSFktRF9ZeUpnUXJBNEgydnZxcmp1NnFteG5tYzhJQkFGWkh4X2xJeXdYNzRnR21jMUZVMFlLMXd0VDhwdURwZEJuNHJZ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sandoz Targets Doubling Sales by 2035 Through Major Biosimilars Expansion</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Major generic and biosimilar manufacturer Sandoz has announced an aggressive strategic push to double its global sales over the next decade by heavily expanding its biosimilars portfolio. This development matters significantly to self-funded employers and benefit managers because a broader market of available biosimilars drives much-needed competition and price compression against expensive biologic reference drugs. For business operations, this signals an accelerating pipeline of affordable alternatives for high-cost specialty medications, presenting substantial opportunities to lower overall healthcare spend and pharmacy benefit costs.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Seeking Alpha</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 09:38:13 GMT</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOUjltSm1QSTYyODE0clVEWnh5VXd4NWhhRmNnbGs0Wl9SSkNFMlN0akl2RDNsc0hBOUdyREdMV1pCRUxaRncyblpEeU1uYVIwYVJmMG5Gbm10a09WUnZ3eDhlVkNHbHgycUVIa29CWnBQeTVHejY4N3lLVWtWTzl2V0NwU2hSNkU1dXh0NHFfaS1tQXA3SnRCbmNzU0hGVC13dmRIOTMwMmR4SmU3UkxqTVBrYTlzQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sandoz Launches Bio 100 Initiative to Expand Biosimilar Portfolio and Drive Market Growth</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sandoz has announced its "Bio 100" strategic initiative, aiming to bring over 100 biosimilars to market by 2040 while doubling sales and achieving a 30%+ EBITDA margin. This aggressive pipeline expansion matters significantly for self-funded employers and pharmacy benefits managers as increased biosimilar competition promises to drive down specialty drug costs and improve affordability. The key business implication is a broader availability of lower-cost alternative biologic therapies, creating new opportunities for plan sponsors to manage high-cost specialty spend effectively over the next decade.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TradingView</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 17:59:18 GMT</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxNdFNBZXRhS0VOR2lhbm5oQXp4d180cGxab3FjQnZlN2RUaW45YVROM0dlMFBpY0dqbzRaVFRmTDE4enE1R0lNeDVPdjVITGJwTTFLLUQ3VnNhVlpQZWN5aFJETm5QUUhQd0R5a2JBZWlWTWVUMTEzeEFCS0NVM3FMbDdXaXlIRWQ2U01WMGd0djVCTG9OajE5NFg3bXpmR1NzT1h3eUs1YVZZT291bFllWWpEbWc1WFlaS29Vd1ZCcm5KeFpIS09YSDhyOUoxd0xDSjVwRmJEaU0yb28waXNSeEJmUkVfTFZ5SENKZXUyYVE5cngzanBleFI0bzNPZlpSYklmXzdwVnlvWkk5?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Investigating The Long-Term Health And Longevity Benefits Of GLP-1 Medications</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Recent discussions highlight the expanding potential of GLP-1 receptor agonists beyond weight loss and diabetes management, exploring their broader impact on overall human longevity and chronic disease prevention. This matters to self-funded employers and pharmacy benefits managers because the widespread adoption of these drugs for longevity could exponentially increase utilization and cost pressures on commercial health plans. Consequently, plan sponsors must carefully evaluate future utilization trends and implement sustainable management strategies to balance employee health outcomes with rising specialty drug expenditures.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SingularityHub</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Tue, 08 Sep 2026 17:33:08 GMT</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPX1J2SVRONm5mYnFBYkNXa1J2SUlXVjF4aHNFTGlWd0h3SDdqRGloNDFFY1pHZlpmUk52SmRBbklwd1EyMzFpRldzeUVMLWxkYWw3QXZ0TnFxb1N3QmdhOGl4MEdPc2FTejFUSk5HODhCZmRXQnNEWlhTSkQ5cmNMUnFIMkM3YTV2NEYxWjZ5aXFpN1pSTjJ4YUln?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Comparative Analysis of 2026 GLP-1 Pricing and Contract Terms Between PlexusDx and ShedRx</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PlexusDx published a direct market comparison evaluating the 2026 pricing structures and contractual terms for GLP-1 medications offered by ShedRx. This comparison sheds light on shifting cost dynamics and vendor terms for high-demand weight-loss therapies entering the commercial landscape. For self-funded employers and pharmacy benefit managers, understanding these evolving market rates is critical for managing surging specialty drug expenditures and designing effective, sustainable benefit plan coverage.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PlexusDx</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Wed, 09 Sep 2026 03:58:54 GMT</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNMEdDdDRrRTdzSE1SemlpOElkeDkxSHRjSlVmZ3NnZVFYbFR6MUV0ZDBkb1lKelJwbUhYWVJGLXdKR1NVeFF3Skl6WkRJVVB0bHN0S0NURWFLOEtZcTktdWpqeFNqS19mM0dhTUg3NDc3OWh2aWxsOER5WUd3U3BxTEN4YV91TkREOEVReUpJZUxtendWeVJyVA?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>